<commit_message>
Data remplacement je l'aime à mourir
</commit_message>
<xml_diff>
--- a/PlaylistInvites.xlsx
+++ b/PlaylistInvites.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="302">
   <si>
     <t>Type</t>
   </si>
@@ -840,9 +840,6 @@
     <t>Je l'aime à mourir</t>
   </si>
   <si>
-    <t>https://music.youtube.com/watch?v=wEsOEtQUHB0</t>
-  </si>
-  <si>
     <t>Despacito</t>
   </si>
   <si>
@@ -919,6 +916,12 @@
   </si>
   <si>
     <t>https://music.youtube.com/watch?v=S_xH7noaqTA</t>
+  </si>
+  <si>
+    <t>Shakira</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/watch?v=R6gHxLmHtIo</t>
   </si>
 </sst>
 </file>
@@ -974,189 +977,7 @@
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="36">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <fill>
         <patternFill>
@@ -3085,10 +2906,10 @@
         <v>273</v>
       </c>
       <c r="G77" t="s">
-        <v>69</v>
+        <v>300</v>
       </c>
       <c r="H77" s="2" t="s">
-        <v>274</v>
+        <v>301</v>
       </c>
     </row>
     <row r="78" spans="3:8" x14ac:dyDescent="0.25">
@@ -3102,13 +2923,13 @@
         <v>4</v>
       </c>
       <c r="F78" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="G78" t="s">
         <v>71</v>
       </c>
       <c r="H78" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="79" spans="3:8" x14ac:dyDescent="0.25">
@@ -3142,18 +2963,18 @@
         <v>4</v>
       </c>
       <c r="F80" t="s">
+        <v>274</v>
+      </c>
+      <c r="G80" t="s">
         <v>275</v>
       </c>
-      <c r="G80" t="s">
+      <c r="H80" s="2" t="s">
         <v>276</v>
-      </c>
-      <c r="H80" s="2" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="81" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C81" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D81" t="s">
         <v>170</v>
@@ -3173,7 +2994,7 @@
     </row>
     <row r="82" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C82" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D82" t="s">
         <v>170</v>
@@ -3182,38 +3003,38 @@
         <v>4</v>
       </c>
       <c r="F82" t="s">
+        <v>280</v>
+      </c>
+      <c r="G82" t="s">
         <v>281</v>
       </c>
-      <c r="G82" t="s">
+      <c r="H82" s="2" t="s">
         <v>282</v>
-      </c>
-      <c r="H82" s="2" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="83" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C83" t="s">
+        <v>283</v>
+      </c>
+      <c r="D83" t="s">
+        <v>168</v>
+      </c>
+      <c r="E83" t="s">
+        <v>3</v>
+      </c>
+      <c r="F83" t="s">
         <v>284</v>
       </c>
-      <c r="D83" t="s">
-        <v>168</v>
-      </c>
-      <c r="E83" t="s">
-        <v>3</v>
-      </c>
-      <c r="F83" t="s">
+      <c r="G83" t="s">
         <v>285</v>
       </c>
-      <c r="G83" t="s">
+      <c r="H83" s="2" t="s">
         <v>286</v>
-      </c>
-      <c r="H83" s="2" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="84" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C84" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D84" t="s">
         <v>168</v>
@@ -3222,18 +3043,18 @@
         <v>3</v>
       </c>
       <c r="F84" t="s">
+        <v>289</v>
+      </c>
+      <c r="G84" t="s">
         <v>290</v>
       </c>
-      <c r="G84" t="s">
+      <c r="H84" s="2" t="s">
         <v>291</v>
-      </c>
-      <c r="H84" s="2" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="85" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C85" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D85" t="s">
         <v>168</v>
@@ -3242,18 +3063,18 @@
         <v>4</v>
       </c>
       <c r="F85" t="s">
+        <v>293</v>
+      </c>
+      <c r="G85" t="s">
         <v>294</v>
       </c>
-      <c r="G85" t="s">
-        <v>295</v>
-      </c>
       <c r="H85" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="86" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C86" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D86" t="s">
         <v>168</v>
@@ -3262,18 +3083,18 @@
         <v>3</v>
       </c>
       <c r="F86" t="s">
+        <v>295</v>
+      </c>
+      <c r="G86" t="s">
         <v>296</v>
       </c>
-      <c r="G86" t="s">
+      <c r="H86" s="2" t="s">
         <v>297</v>
-      </c>
-      <c r="H86" s="2" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="87" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C87" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D87" t="s">
         <v>168</v>
@@ -3282,53 +3103,53 @@
         <v>4</v>
       </c>
       <c r="F87" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G87" t="s">
         <v>255</v>
       </c>
       <c r="H87" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:G77 C78:E81 C82:G104">
-    <cfRule type="expression" dxfId="27" priority="9">
+    <cfRule type="expression" dxfId="9" priority="9">
       <formula>$E2="Coupable"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="10">
+    <cfRule type="expression" dxfId="8" priority="10">
       <formula>$E2="Préférée"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F79:G79">
-    <cfRule type="expression" dxfId="25" priority="5">
+    <cfRule type="expression" dxfId="7" priority="5">
       <formula>$E79="Coupable"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="6">
+    <cfRule type="expression" dxfId="6" priority="6">
       <formula>$E79="Préférée"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F80:G80">
-    <cfRule type="expression" dxfId="23" priority="13">
+    <cfRule type="expression" dxfId="5" priority="13">
       <formula>$E78="Coupable"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="14">
+    <cfRule type="expression" dxfId="4" priority="14">
       <formula>$E78="Préférée"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F78:G78">
-    <cfRule type="expression" dxfId="21" priority="3">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>$E76="Coupable"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="4">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>$E76="Préférée"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F81:G81">
-    <cfRule type="expression" dxfId="11" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>$E81="Coupable"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>$E81="Préférée"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3346,15 +3167,15 @@
     <hyperlink ref="H74" r:id="rId11"/>
     <hyperlink ref="H75" r:id="rId12"/>
     <hyperlink ref="H76" r:id="rId13"/>
-    <hyperlink ref="H77" r:id="rId14"/>
-    <hyperlink ref="H80" r:id="rId15"/>
-    <hyperlink ref="H81" r:id="rId16"/>
-    <hyperlink ref="H82" r:id="rId17"/>
-    <hyperlink ref="H83" r:id="rId18"/>
-    <hyperlink ref="H84" r:id="rId19"/>
-    <hyperlink ref="H85" r:id="rId20"/>
-    <hyperlink ref="H86" r:id="rId21"/>
-    <hyperlink ref="H87" r:id="rId22"/>
+    <hyperlink ref="H80" r:id="rId14"/>
+    <hyperlink ref="H81" r:id="rId15"/>
+    <hyperlink ref="H82" r:id="rId16"/>
+    <hyperlink ref="H83" r:id="rId17"/>
+    <hyperlink ref="H84" r:id="rId18"/>
+    <hyperlink ref="H85" r:id="rId19"/>
+    <hyperlink ref="H86" r:id="rId20"/>
+    <hyperlink ref="H87" r:id="rId21"/>
+    <hyperlink ref="H77" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId23"/>

</xml_diff>